<commit_message>
success read from excel
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/PythonProject/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA212B00-6A2E-4B48-A058-B51D671E468C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CAC847E-B185-9445-B394-7FDA491BA2DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="21260" xr2:uid="{522619BB-B2B9-E146-AC0C-62816396454E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>nik</t>
   </si>
@@ -84,6 +84,54 @@
   </si>
   <si>
     <t>1982-05-22</t>
+  </si>
+  <si>
+    <t>Belum Menikah</t>
+  </si>
+  <si>
+    <t>pernikahan</t>
+  </si>
+  <si>
+    <t>pekerjaan</t>
+  </si>
+  <si>
+    <t>Pegawai Swasta</t>
+  </si>
+  <si>
+    <t>prov</t>
+  </si>
+  <si>
+    <t>kab</t>
+  </si>
+  <si>
+    <t>kec</t>
+  </si>
+  <si>
+    <t>desa</t>
+  </si>
+  <si>
+    <t>domisili</t>
+  </si>
+  <si>
+    <t>Jawa Timur</t>
+  </si>
+  <si>
+    <t>Kab. Situbondo</t>
+  </si>
+  <si>
+    <t>Kendit</t>
+  </si>
+  <si>
+    <t>Balung</t>
+  </si>
+  <si>
+    <t>Jl. ABCD</t>
+  </si>
+  <si>
+    <t>3512052205820001</t>
+  </si>
+  <si>
+    <t>3509053001929991</t>
   </si>
 </sst>
 </file>
@@ -456,10 +504,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{522244BB-2C32-6B42-AC05-1B00C4A8A02B}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.5" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
@@ -467,10 +515,11 @@
     <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.83203125" style="1"/>
     <col min="9" max="9" width="10.83203125" style="1"/>
-    <col min="11" max="11" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -504,10 +553,31 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" t="s">
+        <v>21</v>
+      </c>
+      <c r="P1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>23</v>
+      </c>
+      <c r="R1" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>3509053001929990</v>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>31</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -524,8 +594,8 @@
       <c r="F2">
         <v>26</v>
       </c>
-      <c r="G2" s="1">
-        <v>3512052205820000</v>
+      <c r="G2" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="H2" t="s">
         <v>14</v>
@@ -538,9 +608,31 @@
       </c>
       <c r="K2">
         <v>81234567890</v>
+      </c>
+      <c r="L2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M2" t="s">
+        <v>19</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+      <c r="O2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>28</v>
+      </c>
+      <c r="R2" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
need patching on tgl_lahir
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="181029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -570,7 +570,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>2010-10-01</t>
+          <t>1998-04-01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
wip tgl_lahir only iterate 3 times
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -565,12 +565,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Bambang</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>1998-01-01</t>
+          <t>1980-10-01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -644,13 +644,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAILED: Locator.click: Target page, context or browser has been closed
-Call log:
-  - waiting for locator(".mx-datepicker-popup").locator(".mx-btn-icon-double-left")
-    - locator resolved to &lt;button type="button" class="mx-btn mx-btn-text mx-btn-icon-double-left"&gt;…&lt;/button&gt;
-  - attempting click action
-    - waiting for element to be visible, enabled and stable
-</t>
+          <t>FAILED: 'Agt'</t>
         </is>
       </c>
     </row>
@@ -662,12 +656,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Franca Milena</t>
+          <t>Yuni</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>1990-03-01</t>
+          <t>1990-12-01</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -741,7 +735,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>FAILED: Page.goto: Target page, context or browser has been closed</t>
+          <t>FAILED: 'Agt'</t>
         </is>
       </c>
     </row>
@@ -753,12 +747,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Siti Supina</t>
+          <t>Dewi Puji</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>1998-08-01</t>
+          <t>1990-05-01</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -832,7 +826,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>FAILED: Page.goto: Target page, context or browser has been closed</t>
+          <t>SUCCESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
done fixing tgl lahir wali
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4D4261-1401-164C-BABF-8C25E3A47712}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B49B9DA0-4354-4549-A7DF-F6317AFBBDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="21260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="40">
   <si>
     <t>nik</t>
   </si>
@@ -136,7 +136,10 @@
     <t>Dewi Puji</t>
   </si>
   <si>
-    <t>1990-05-01</t>
+    <t>SUCCESS</t>
+  </si>
+  <si>
+    <t>1990-06-01</t>
   </si>
 </sst>
 </file>
@@ -638,6 +641,9 @@
       <c r="R2" t="s">
         <v>31</v>
       </c>
+      <c r="S2" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -694,6 +700,9 @@
       <c r="R3" t="s">
         <v>31</v>
       </c>
+      <c r="S3" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -703,7 +712,7 @@
         <v>37</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
         <v>35</v>

</xml_diff>